<commit_message>
docs: change security status reporting terminology from Remediated to Pass/Fail
</commit_message>
<xml_diff>
--- a/Vulnerability Test Results/endpoint-inventory.xlsx
+++ b/Vulnerability Test Results/endpoint-inventory.xlsx
@@ -509,7 +509,7 @@
     <col width="40" customWidth="1" min="7" max="7"/>
     <col width="40" customWidth="1" min="8" max="8"/>
     <col width="40" customWidth="1" min="9" max="9"/>
-    <col width="13" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1" ht="25" customHeight="1">
@@ -612,7 +612,7 @@
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>Remediated</t>
+          <t>Pass</t>
         </is>
       </c>
     </row>
@@ -664,7 +664,7 @@
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>Remediated</t>
+          <t>Pass</t>
         </is>
       </c>
     </row>
@@ -716,7 +716,7 @@
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>Remediated</t>
+          <t>Pass</t>
         </is>
       </c>
     </row>
@@ -768,7 +768,7 @@
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>Remediated</t>
+          <t>Pass</t>
         </is>
       </c>
     </row>
@@ -820,7 +820,7 @@
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>Remediated</t>
+          <t>Pass</t>
         </is>
       </c>
     </row>
@@ -872,7 +872,7 @@
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>Remediated</t>
+          <t>Pass</t>
         </is>
       </c>
     </row>
@@ -1581,8 +1581,8 @@
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
     <col width="19" customWidth="1" min="2" max="2"/>
-    <col width="13" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1" ht="25" customHeight="1">
@@ -1598,12 +1598,12 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Remediated</t>
+          <t>Pass</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Residual Risk</t>
+          <t>Fail</t>
         </is>
       </c>
     </row>

</xml_diff>